<commit_message>
Module 2: acts injection via skill
</commit_message>
<xml_diff>
--- a/plan-vs-fact.xlsx
+++ b/plan-vs-fact.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Сводка'!$A$1:$J$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Детализация'!$A$1:$F$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Детализация'!$A$1:$F$116</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Данные_доходы'!$A$1:$F$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -828,7 +828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F112"/>
+  <dimension ref="A1:F116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2022,29 +2022,29 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>PRJ-2026-003</t>
+          <t>PRJ-2026-002</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Цифровая платформа 2.0</t>
+          <t>Региональная программа — Сибирь</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>IT-инфраструктура</t>
+          <t>Расчёты с подрядчиками</t>
         </is>
       </c>
       <c r="E43" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>1800</v>
+        <v>950</v>
       </c>
     </row>
     <row r="44">
@@ -2065,14 +2065,14 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Инфраструктура / IT</t>
+          <t>IT-инфраструктура</t>
         </is>
       </c>
       <c r="E44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="3" t="n">
         <v>1800</v>
-      </c>
-      <c r="F44" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -2093,14 +2093,14 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Маркетинг</t>
+          <t>Инфраструктура / IT</t>
         </is>
       </c>
       <c r="E45" s="3" t="n">
-        <v>0</v>
+        <v>1800</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>220</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -2121,14 +2121,14 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Маркетинг (анонс релиза)</t>
+          <t>Маркетинг</t>
         </is>
       </c>
       <c r="E46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="3" t="n">
         <v>220</v>
-      </c>
-      <c r="F46" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -2149,14 +2149,14 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Оплата труда</t>
+          <t>Маркетинг (анонс релиза)</t>
         </is>
       </c>
       <c r="E47" s="3" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>4640</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -2177,14 +2177,14 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Подрядчики (дизайн, интеграции)</t>
+          <t>Оплата труда</t>
         </is>
       </c>
       <c r="E48" s="3" t="n">
-        <v>1100</v>
+        <v>0</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>0</v>
+        <v>4640</v>
       </c>
     </row>
     <row r="49">
@@ -2205,14 +2205,14 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Производство контента</t>
+          <t>Подрядчики (дизайн, интеграции)</t>
         </is>
       </c>
       <c r="E49" s="3" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>380</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -2233,14 +2233,14 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Производство контента (релизный)</t>
+          <t>Производство контента</t>
         </is>
       </c>
       <c r="E50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="3" t="n">
         <v>380</v>
-      </c>
-      <c r="F50" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -2261,11 +2261,11 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Прочее (юр-блок, аудит)</t>
+          <t>Производство контента (релизный)</t>
         </is>
       </c>
       <c r="E51" s="3" t="n">
-        <v>240</v>
+        <v>380</v>
       </c>
       <c r="F51" s="3" t="n">
         <v>0</v>
@@ -2289,14 +2289,14 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Прочие расходы</t>
+          <t>Прочее (юр-блок, аудит)</t>
         </is>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>240</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -2317,14 +2317,14 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Расчёты с подрядчиками</t>
+          <t>Прочие расходы</t>
         </is>
       </c>
       <c r="E53" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>1100</v>
+        <v>240</v>
       </c>
     </row>
     <row r="54">
@@ -2345,14 +2345,14 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>ФОТ</t>
+          <t>Расчёты с подрядчиками</t>
         </is>
       </c>
       <c r="E54" s="3" t="n">
-        <v>4500</v>
+        <v>0</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="55">
@@ -2368,19 +2368,19 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>IT-инфраструктура</t>
+          <t>ФОТ</t>
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>0</v>
+        <v>4500</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -2401,14 +2401,14 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Инфраструктура / IT</t>
+          <t>IT-инфраструктура</t>
         </is>
       </c>
       <c r="E56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="3" t="n">
         <v>600</v>
-      </c>
-      <c r="F56" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -2429,14 +2429,14 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Маркетинг</t>
+          <t>Инфраструктура / IT</t>
         </is>
       </c>
       <c r="E57" s="3" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>280</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -2457,14 +2457,14 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Маркетинг (анонс релиза)</t>
+          <t>Маркетинг</t>
         </is>
       </c>
       <c r="E58" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="3" t="n">
         <v>280</v>
-      </c>
-      <c r="F58" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -2485,14 +2485,14 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Оплата труда</t>
+          <t>Маркетинг (анонс релиза)</t>
         </is>
       </c>
       <c r="E59" s="3" t="n">
-        <v>0</v>
+        <v>280</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>4640</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -2513,14 +2513,14 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Подрядчики (дизайн, интеграции)</t>
+          <t>Оплата труда</t>
         </is>
       </c>
       <c r="E60" s="3" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>0</v>
+        <v>4640</v>
       </c>
     </row>
     <row r="61">
@@ -2541,14 +2541,14 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Производство контента</t>
+          <t>Подрядчики (дизайн, интеграции)</t>
         </is>
       </c>
       <c r="E61" s="3" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>380</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -2569,14 +2569,14 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Производство контента (релизный)</t>
+          <t>Производство контента</t>
         </is>
       </c>
       <c r="E62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" s="3" t="n">
         <v>380</v>
-      </c>
-      <c r="F62" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -2597,11 +2597,11 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Прочее (юр-блок, аудит)</t>
+          <t>Производство контента (релизный)</t>
         </is>
       </c>
       <c r="E63" s="3" t="n">
-        <v>200</v>
+        <v>380</v>
       </c>
       <c r="F63" s="3" t="n">
         <v>0</v>
@@ -2625,14 +2625,14 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Прочие расходы</t>
+          <t>Прочее (юр-блок, аудит)</t>
         </is>
       </c>
       <c r="E64" s="3" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -2653,14 +2653,14 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Расчёты с подрядчиками</t>
+          <t>Прочие расходы</t>
         </is>
       </c>
       <c r="E65" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>4000</v>
+        <v>200</v>
       </c>
     </row>
     <row r="66">
@@ -2681,14 +2681,14 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>ФОТ</t>
+          <t>Расчёты с подрядчиками</t>
         </is>
       </c>
       <c r="E66" s="3" t="n">
-        <v>4600</v>
+        <v>0</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="67">
@@ -2704,19 +2704,19 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>IT-инфраструктура</t>
+          <t>ФОТ</t>
         </is>
       </c>
       <c r="E67" s="3" t="n">
-        <v>0</v>
+        <v>4600</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -2737,14 +2737,14 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Инфраструктура / IT</t>
+          <t>IT-инфраструктура</t>
         </is>
       </c>
       <c r="E68" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" s="3" t="n">
         <v>800</v>
-      </c>
-      <c r="F68" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -2765,14 +2765,14 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Маркетинг</t>
+          <t>Инфраструктура / IT</t>
         </is>
       </c>
       <c r="E69" s="3" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -2793,14 +2793,14 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Маркетинг (анонс релиза)</t>
+          <t>Маркетинг</t>
         </is>
       </c>
       <c r="E70" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" s="3" t="n">
         <v>800</v>
-      </c>
-      <c r="F70" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -2821,14 +2821,14 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Оплата труда</t>
+          <t>Маркетинг (анонс релиза)</t>
         </is>
       </c>
       <c r="E71" s="3" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="F71" s="3" t="n">
-        <v>4530</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -2849,14 +2849,14 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Подрядчики (дизайн, интеграции)</t>
+          <t>Оплата труда</t>
         </is>
       </c>
       <c r="E72" s="3" t="n">
-        <v>1700</v>
+        <v>0</v>
       </c>
       <c r="F72" s="3" t="n">
-        <v>0</v>
+        <v>4530</v>
       </c>
     </row>
     <row r="73">
@@ -2877,14 +2877,14 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Производство контента</t>
+          <t>Подрядчики (дизайн, интеграции)</t>
         </is>
       </c>
       <c r="E73" s="3" t="n">
-        <v>0</v>
+        <v>1700</v>
       </c>
       <c r="F73" s="3" t="n">
-        <v>380</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -2905,14 +2905,14 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Производство контента (релизный)</t>
+          <t>Производство контента</t>
         </is>
       </c>
       <c r="E74" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="3" t="n">
         <v>380</v>
-      </c>
-      <c r="F74" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Прочее (юр-блок, аудит)</t>
+          <t>Производство контента (релизный)</t>
         </is>
       </c>
       <c r="E75" s="3" t="n">
-        <v>360</v>
+        <v>380</v>
       </c>
       <c r="F75" s="3" t="n">
         <v>0</v>
@@ -2961,14 +2961,14 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Прочие расходы</t>
+          <t>Прочее (юр-блок, аудит)</t>
         </is>
       </c>
       <c r="E76" s="3" t="n">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -2989,14 +2989,14 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Расчёты с подрядчиками</t>
+          <t>Прочие расходы</t>
         </is>
       </c>
       <c r="E77" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F77" s="3" t="n">
-        <v>1700</v>
+        <v>360</v>
       </c>
     </row>
     <row r="78">
@@ -3017,114 +3017,114 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>ФОТ</t>
+          <t>Расчёты с подрядчиками</t>
         </is>
       </c>
       <c r="E78" s="3" t="n">
-        <v>4700</v>
+        <v>0</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>0</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>PRJ-2026-004</t>
+          <t>PRJ-2026-003</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>B2B со Сбером</t>
+          <t>Цифровая платформа 2.0</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Оплата труда</t>
+          <t>ФОТ</t>
         </is>
       </c>
       <c r="E79" s="3" t="n">
-        <v>0</v>
+        <v>4700</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>1560</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>PRJ-2026-004</t>
+          <t>PRJ-2026-003</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>B2B со Сбером</t>
+          <t>Цифровая платформа 2.0</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Подрядчики (методология для B2B)</t>
+          <t>IT-инфраструктура</t>
         </is>
       </c>
       <c r="E80" s="3" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>0</v>
+        <v>620</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>PRJ-2026-004</t>
+          <t>PRJ-2026-003</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>B2B со Сбером</t>
+          <t>Цифровая платформа 2.0</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Прочие расходы</t>
+          <t>Маркетинг</t>
         </is>
       </c>
       <c r="E81" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F81" s="3" t="n">
-        <v>300</v>
+        <v>440</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>PRJ-2026-004</t>
+          <t>PRJ-2026-003</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>B2B со Сбером</t>
+          <t>Цифровая платформа 2.0</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -3136,7 +3136,7 @@
         <v>0</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>620</v>
+        <v>940</v>
       </c>
     </row>
     <row r="83">
@@ -3157,14 +3157,14 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>ФОТ</t>
+          <t>Оплата труда</t>
         </is>
       </c>
       <c r="E83" s="3" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="F83" s="3" t="n">
-        <v>0</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="84">
@@ -3185,11 +3185,11 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Юр-блок (B2B-сопровождение)</t>
+          <t>Подрядчики (методология для B2B)</t>
         </is>
       </c>
       <c r="E84" s="3" t="n">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="F84" s="3" t="n">
         <v>0</v>
@@ -3208,19 +3208,19 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Оплата труда</t>
+          <t>Прочие расходы</t>
         </is>
       </c>
       <c r="E85" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F85" s="3" t="n">
-        <v>1560</v>
+        <v>300</v>
       </c>
     </row>
     <row r="86">
@@ -3236,19 +3236,19 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Подрядчики (методология для B2B)</t>
+          <t>Расчёты с подрядчиками</t>
         </is>
       </c>
       <c r="E86" s="3" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>0</v>
+        <v>620</v>
       </c>
     </row>
     <row r="87">
@@ -3264,19 +3264,19 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Прочие расходы</t>
+          <t>ФОТ</t>
         </is>
       </c>
       <c r="E87" s="3" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -3292,19 +3292,19 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Расчёты с подрядчиками</t>
+          <t>Юр-блок (B2B-сопровождение)</t>
         </is>
       </c>
       <c r="E88" s="3" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89">
@@ -3325,14 +3325,14 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>ФОТ</t>
+          <t>Оплата труда</t>
         </is>
       </c>
       <c r="E89" s="3" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>0</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="90">
@@ -3353,11 +3353,11 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Юр-блок (B2B-сопровождение)</t>
+          <t>Подрядчики (методология для B2B)</t>
         </is>
       </c>
       <c r="E90" s="3" t="n">
-        <v>400</v>
+        <v>800</v>
       </c>
       <c r="F90" s="3" t="n">
         <v>0</v>
@@ -3376,19 +3376,19 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Оплата труда</t>
+          <t>Прочие расходы</t>
         </is>
       </c>
       <c r="E91" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F91" s="3" t="n">
-        <v>1560</v>
+        <v>400</v>
       </c>
     </row>
     <row r="92">
@@ -3404,19 +3404,19 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Подрядчики (методология для B2B)</t>
+          <t>Расчёты с подрядчиками</t>
         </is>
       </c>
       <c r="E92" s="3" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
     </row>
     <row r="93">
@@ -3432,19 +3432,19 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Прочие расходы</t>
+          <t>ФОТ</t>
         </is>
       </c>
       <c r="E93" s="3" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="F93" s="3" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -3460,19 +3460,19 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Расчёты с подрядчиками</t>
+          <t>Юр-блок (B2B-сопровождение)</t>
         </is>
       </c>
       <c r="E94" s="3" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -3493,14 +3493,14 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>ФОТ</t>
+          <t>Оплата труда</t>
         </is>
       </c>
       <c r="E95" s="3" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>0</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="96">
@@ -3521,11 +3521,11 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Юр-блок (B2B-сопровождение)</t>
+          <t>Подрядчики (методология для B2B)</t>
         </is>
       </c>
       <c r="E96" s="3" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="F96" s="3" t="n">
         <v>0</v>
@@ -3534,82 +3534,82 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>PRJ-2026-005</t>
+          <t>PRJ-2026-004</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Аудиокниги — летний релиз</t>
+          <t>B2B со Сбером</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Запись аудиокниг (студия)</t>
+          <t>Прочие расходы</t>
         </is>
       </c>
       <c r="E97" s="3" t="n">
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>PRJ-2026-005</t>
+          <t>PRJ-2026-004</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Аудиокниги — летний релиз</t>
+          <t>B2B со Сбером</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Оплата труда</t>
+          <t>Расчёты с подрядчиками</t>
         </is>
       </c>
       <c r="E98" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>720</v>
+        <v>500</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>PRJ-2026-005</t>
+          <t>PRJ-2026-004</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Аудиокниги — летний релиз</t>
+          <t>B2B со Сбером</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Постпродакшн</t>
+          <t>ФОТ</t>
         </is>
       </c>
       <c r="E99" s="3" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="F99" s="3" t="n">
         <v>0</v>
@@ -3618,29 +3618,29 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>PRJ-2026-005</t>
+          <t>PRJ-2026-004</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Аудиокниги — летний релиз</t>
+          <t>B2B со Сбером</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Расчёты с подрядчиками</t>
+          <t>Юр-блок (B2B-сопровождение)</t>
         </is>
       </c>
       <c r="E100" s="3" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="F100" s="3" t="n">
-        <v>700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -3661,7 +3661,7 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>ФОТ</t>
+          <t>Запись аудиокниг (студия)</t>
         </is>
       </c>
       <c r="E101" s="3" t="n">
@@ -3684,19 +3684,19 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Запись аудиокниг (студия)</t>
+          <t>Оплата труда</t>
         </is>
       </c>
       <c r="E102" s="3" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>0</v>
+        <v>720</v>
       </c>
     </row>
     <row r="103">
@@ -3712,19 +3712,19 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Оплата труда</t>
+          <t>Постпродакшн</t>
         </is>
       </c>
       <c r="E103" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F103" s="3" t="n">
-        <v>720</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104">
@@ -3740,19 +3740,19 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Постпродакшн</t>
+          <t>Расчёты с подрядчиками</t>
         </is>
       </c>
       <c r="E104" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F104" s="3" t="n">
-        <v>0</v>
+        <v>700</v>
       </c>
     </row>
     <row r="105">
@@ -3768,19 +3768,19 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>Расчёты с подрядчиками</t>
+          <t>ФОТ</t>
         </is>
       </c>
       <c r="E105" s="3" t="n">
-        <v>0</v>
+        <v>700</v>
       </c>
       <c r="F105" s="3" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106">
@@ -3801,11 +3801,11 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>ФОТ</t>
+          <t>Запись аудиокниг (студия)</t>
         </is>
       </c>
       <c r="E106" s="3" t="n">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="F106" s="3" t="n">
         <v>0</v>
@@ -3824,19 +3824,19 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Запись аудиокниг (студия)</t>
+          <t>Оплата труда</t>
         </is>
       </c>
       <c r="E107" s="3" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="F107" s="3" t="n">
-        <v>0</v>
+        <v>720</v>
       </c>
     </row>
     <row r="108">
@@ -3852,19 +3852,19 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Оплата труда</t>
+          <t>Постпродакшн</t>
         </is>
       </c>
       <c r="E108" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F108" s="3" t="n">
-        <v>620</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109">
@@ -3880,19 +3880,19 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Постпродакшн</t>
+          <t>Расчёты с подрядчиками</t>
         </is>
       </c>
       <c r="E109" s="3" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="F109" s="3" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
     </row>
     <row r="110">
@@ -3908,19 +3908,19 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Производство контента</t>
+          <t>ФОТ</t>
         </is>
       </c>
       <c r="E110" s="3" t="n">
-        <v>0</v>
+        <v>700</v>
       </c>
       <c r="F110" s="3" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111">
@@ -3941,14 +3941,14 @@
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Расчёты с подрядчиками</t>
+          <t>Запись аудиокниг (студия)</t>
         </is>
       </c>
       <c r="E111" s="3" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="F111" s="3" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112">
@@ -3969,18 +3969,130 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
+          <t>Оплата труда</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F112" s="3" t="n">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>PRJ-2026-005</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>Аудиокниги — летний релиз</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>Постпродакшн</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="F113" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>PRJ-2026-005</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Аудиокниги — летний релиз</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>Производство контента</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F114" s="3" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>PRJ-2026-005</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Аудиокниги — летний релиз</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>Расчёты с подрядчиками</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F115" s="3" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>PRJ-2026-005</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Аудиокниги — летний релиз</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
           <t>ФОТ</t>
         </is>
       </c>
-      <c r="E112" s="3" t="n">
+      <c r="E116" s="3" t="n">
         <v>600</v>
       </c>
-      <c r="F112" s="3" t="n">
+      <c r="F116" s="3" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F112"/>
+  <autoFilter ref="A1:F116"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>